<commit_message>
Refresh precedents template (analyst follow-up); v1.9.10
Replaces INFOR Precedents Template.xlsx with the latest analyst-updated
workbook. Cell references and write rules are unchanged — same 15-row
layout (rows 7-21) with averages at row 23 — so no SKILL workflow edits
are needed beyond the version bump.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/infor-workflows/templates/INFOR Precedents Template.xlsx
+++ b/infor-workflows/templates/INFOR Precedents Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude - INFOR/infor-workflows/infor-workflows/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="274" documentId="8_{0848B0FA-4984-42F6-80CF-A7F512337903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00EB3BDD-D27A-4E64-A7E5-64DB8C62CC7E}"/>
+  <xr:revisionPtr revIDLastSave="295" documentId="8_{0848B0FA-4984-42F6-80CF-A7F512337903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E5C2B7A-2DC3-457F-9D88-CB60E96CFB41}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{A6BB75E0-A801-473C-9678-28D65ECCDC5E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{A6BB75E0-A801-473C-9678-28D65ECCDC5E}"/>
   </bookViews>
   <sheets>
     <sheet name="__snloffice" sheetId="2" state="veryHidden" r:id="rId1"/>
@@ -131,9 +131,6 @@
     <t>Average</t>
   </si>
   <si>
-    <t>允䅁䅁䅣䅁敁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䍁䅁杔䉂䑁䄰杔䉂䅁䅁杁䅁䉁䅁䅁歁䕁䅍兑䕂䕁䅣村兂䅁䅁䅁䅁䉁䅁䅁歁䕁䅍兑䕂䙁䅕睕䕂䅁䅁睁䅁䉁䄴䅁呂䙁䅁睘兂䙁䅉兓䑂䕁䅕睘䑂䕁䅷睔呂䕁䅕䅁䉁䅁䅁䅏䅁䍁䅍兓佂䙁䅙兑䵂䕁䅫䅒杁䕁䅙兖佂䕁䅍䅖䩂䕁䄸杔杁䙁䅁兑卂䕁䅅兔䙂䙁䅑兒卂䅁䅁兂䅁䉁䅑䅁歁䕁䅍兑䕂䑁䅑李睁䑁䅉睍䅁䅁䅑䅁允䅁䅁䅊䑂䕁䅅䅒䑂䕁䅅䅒䅁䅁䅙䅁䅁䅁䅁</t>
-  </si>
-  <si>
     <t xml:space="preserve">TEV </t>
   </si>
   <si>
@@ -144,6 +141,9 @@
   </si>
   <si>
     <t>Ann. Date</t>
+  </si>
+  <si>
+    <t>允䅁䅁䅫䅁允䅁䅁䅊䑂䕁䅅䅒䡂䕁䅉䅕䅁䅁䅁䅁敁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䍁䅁杔䉂䑁䄰杔䉂䅁䅁杁䅁䉁䄴䅁呂䙁䅁睘兂䙁䅉兓䑂䕁䅕睘䑂䕁䅷睔呂䕁䅕䅁䉁䅁䅁䅅䅁䍁䅑睑䉂䕁䅑兖呂䕁䅑䅁䑁䅁䅁䅆䅁䍁䅑睑䉂䕁䅑䅎㉁䑁䅁杍穁䅁䅁䅂䅁䑁䅧䅁橁䕁䅫杔坂䕁䅅䅔䩂䕁䅑䅉䝂䙁䅕杔䑂䙁䅑兓偂䕁䄴䅉兂䕁䅅杕䉂䕁䄰兒啂䕁䅕杕䅁䅁䅕䅁允䅁䅁䅊䑂䕁䅅䅒䑂䕁䅅䅒䅁䅁䅙䅁䭁䅁䅁䅊䑂䕁䅅䅒䅁䅁䅣䅁潁䅁䅁睉䩂䕁䄴杖䉂䕁䅷兓䕂䍁䅁睑偂䕁䄰䅕䉂䕁䄴兗杁䕁䅫䅒䅁䅁䅧䅁䑁䅁䅁䍄䉁䅁䅁兂䅁䅁䅍䅄䅁䅁䅯睂䅁䅁䅯允䅁䅁䅕䅁䅁佁㑂欵䭁䅁䅉䅁䉁䅁䅁允䅁䅁䅯䅃䅁䅁杷允䅁䅁䅕䅁䑁䅁䅷䅁䭁䅁䅣䅁䭁䅁䅅䅁䭁偁䡑潃䭁䅁䅉䅁䉁䅁䅁允䅁䅁䅯兂䅁䅁杷允䅁䅁䅕䅁䑁䅁䅷䅁䭁䅁䅙䅁䭁䅁䅅䅁䙁䅁䅁䅁杄佥䅚权䍁䅁䅁允䅁䅁䅅䅁啁䅁䅅䅁䅁䅁䅁</t>
   </si>
 </sst>
 </file>
@@ -389,9 +389,6 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="15" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -433,6 +430,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -774,7 +774,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -817,7 +817,7 @@
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="33" t="str">
+      <c r="E4" s="32" t="str">
         <f>"Figures in "&amp;IF($H$2="CAD","C$MM","US$MM")</f>
         <v>Figures in C$MM</v>
       </c>
@@ -828,10 +828,10 @@
       <c r="J4" s="8"/>
       <c r="K4" s="8"/>
       <c r="L4" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N4" s="8"/>
     </row>
@@ -843,7 +843,7 @@
         <v>11</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>2</v>
@@ -864,10 +864,10 @@
         <v>4</v>
       </c>
       <c r="L5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="M5" s="8" t="s">
         <v>16</v>
-      </c>
-      <c r="M5" s="8" t="s">
-        <v>17</v>
       </c>
       <c r="N5" s="12" t="s">
         <v>12</v>
@@ -875,372 +875,372 @@
     </row>
     <row r="6" spans="2:14" customFormat="1" ht="3" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B7" s="21"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="11" t="str" cm="1">
-        <f t="array" ref="C7">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B7,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
-      </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="24" t="str">
+        <f t="array" ref="C7">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B7,"SP_PRICE_CLOSE",WORKDAY(E7+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
+      </c>
+      <c r="E7" s="33"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="23" t="str">
         <f>IFERROR($I7/J7,"n/a ")</f>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M7" s="24" t="str">
+      <c r="M7" s="23" t="str">
         <f>IFERROR($I7/K7,"n/a ")</f>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="N7" s="20"/>
+      <c r="N7" s="19"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B8" s="21"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="11" t="str" cm="1">
-        <f t="array" ref="C8">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B8,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C8">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B8,"SP_PRICE_CLOSE",WORKDAY(E8+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E8" s="13"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
       <c r="H8" s="15"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="25" t="str">
+      <c r="I8" s="29"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="24" t="str">
         <f t="shared" ref="L8:L21" si="0">IFERROR($I8/J8,"n/a ")</f>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M8" s="25" t="str">
+      <c r="M8" s="24" t="str">
         <f t="shared" ref="M8:M21" si="1">IFERROR($I8/K8,"n/a ")</f>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N8" s="16"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B9" s="21"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="11" t="str" cm="1">
-        <f t="array" ref="C9">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B9,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C9">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B9,"SP_PRICE_CLOSE",WORKDAY(E9+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E9" s="13"/>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="15"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="25" t="str">
+      <c r="I9" s="29"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M9" s="25" t="str">
+      <c r="M9" s="24" t="str">
         <f t="shared" si="1"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N9" s="16"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B10" s="21"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="11" t="str" cm="1">
-        <f t="array" ref="C10">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B10,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C10">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B10,"SP_PRICE_CLOSE",WORKDAY(E10+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E10" s="13"/>
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
       <c r="H10" s="15"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="25" t="str">
+      <c r="I10" s="29"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M10" s="25" t="str">
+      <c r="M10" s="24" t="str">
         <f t="shared" si="1"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N10" s="16"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B11" s="21"/>
+      <c r="B11" s="20"/>
       <c r="C11" s="11" t="str" cm="1">
-        <f t="array" ref="C11">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B11,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C11">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B11,"SP_PRICE_CLOSE",WORKDAY(E11+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E11" s="13"/>
       <c r="F11" s="14"/>
       <c r="G11" s="14"/>
       <c r="H11" s="15"/>
-      <c r="I11" s="30"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="25" t="str">
+      <c r="I11" s="29"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="22"/>
+      <c r="L11" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M11" s="25" t="str">
+      <c r="M11" s="24" t="str">
         <f t="shared" si="1"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N11" s="16"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="11" t="str" cm="1">
-        <f t="array" ref="C12">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B12,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C12">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B12,"SP_PRICE_CLOSE",WORKDAY(E12+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="14"/>
       <c r="G12" s="14"/>
       <c r="H12" s="15"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="23"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="25" t="str">
+      <c r="I12" s="29"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="22"/>
+      <c r="L12" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M12" s="25" t="str">
+      <c r="M12" s="24" t="str">
         <f t="shared" si="1"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N12" s="16"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="21"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="11" t="str" cm="1">
-        <f t="array" ref="C13">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B13,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C13">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B13,"SP_PRICE_CLOSE",WORKDAY(E13+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E13" s="13"/>
       <c r="F13" s="14"/>
       <c r="G13" s="14"/>
       <c r="H13" s="15"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="25" t="str">
+      <c r="I13" s="29"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M13" s="25" t="str">
+      <c r="M13" s="24" t="str">
         <f t="shared" si="1"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N13" s="16"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
+      <c r="B14" s="20"/>
       <c r="C14" s="11" t="str" cm="1">
-        <f t="array" ref="C14">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B14,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C14">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B14,"SP_PRICE_CLOSE",WORKDAY(E14+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E14" s="13"/>
       <c r="F14" s="14"/>
       <c r="G14" s="14"/>
       <c r="H14" s="15"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="25" t="str">
+      <c r="I14" s="29"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="22"/>
+      <c r="L14" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M14" s="25" t="str">
+      <c r="M14" s="24" t="str">
         <f t="shared" ref="M14:M20" si="2">IFERROR($I14/K14,"n/a ")</f>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N14" s="16"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
+      <c r="B15" s="20"/>
       <c r="C15" s="11" t="str" cm="1">
-        <f t="array" ref="C15">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B15,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C15">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B15,"SP_PRICE_CLOSE",WORKDAY(E15+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E15" s="13"/>
       <c r="F15" s="14"/>
       <c r="G15" s="14"/>
       <c r="H15" s="15"/>
-      <c r="I15" s="30"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="25" t="str">
+      <c r="I15" s="29"/>
+      <c r="J15" s="22"/>
+      <c r="K15" s="22"/>
+      <c r="L15" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M15" s="25" t="str">
+      <c r="M15" s="24" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N15" s="16"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
+      <c r="B16" s="20"/>
       <c r="C16" s="11" t="str" cm="1">
-        <f t="array" ref="C16">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B16,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C16">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B16,"SP_PRICE_CLOSE",WORKDAY(E16+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E16" s="13"/>
       <c r="F16" s="14"/>
       <c r="G16" s="14"/>
       <c r="H16" s="15"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="25" t="str">
+      <c r="I16" s="29"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M16" s="25" t="str">
+      <c r="M16" s="24" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N16" s="16"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B17" s="21"/>
+      <c r="B17" s="20"/>
       <c r="C17" s="11" t="str" cm="1">
-        <f t="array" ref="C17">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B17,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C17">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B17,"SP_PRICE_CLOSE",WORKDAY(E17+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E17" s="13"/>
       <c r="F17" s="14"/>
       <c r="G17" s="14"/>
       <c r="H17" s="15"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="25" t="str">
+      <c r="I17" s="29"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M17" s="25" t="str">
+      <c r="M17" s="24" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N17" s="16"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B18" s="21"/>
+      <c r="B18" s="20"/>
       <c r="C18" s="11" t="str" cm="1">
-        <f t="array" ref="C18">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B18,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C18">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B18,"SP_PRICE_CLOSE",WORKDAY(E18+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E18" s="13"/>
       <c r="F18" s="14"/>
       <c r="G18" s="14"/>
       <c r="H18" s="15"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="23"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="25" t="str">
+      <c r="I18" s="29"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M18" s="25" t="str">
+      <c r="M18" s="24" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N18" s="16"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B19" s="21"/>
+      <c r="B19" s="20"/>
       <c r="C19" s="11" t="str" cm="1">
-        <f t="array" ref="C19">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B19,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C19">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B19,"SP_PRICE_CLOSE",WORKDAY(E19+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E19" s="13"/>
       <c r="F19" s="14"/>
       <c r="G19" s="14"/>
       <c r="H19" s="15"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="25" t="str">
+      <c r="I19" s="29"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M19" s="25" t="str">
+      <c r="M19" s="24" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N19" s="16"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B20" s="21"/>
+      <c r="B20" s="20"/>
       <c r="C20" s="11" t="str" cm="1">
-        <f t="array" ref="C20">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B20,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C20">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B20,"SP_PRICE_CLOSE",WORKDAY(E20+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="14"/>
       <c r="G20" s="14"/>
       <c r="H20" s="15"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="25" t="str">
+      <c r="I20" s="29"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M20" s="25" t="str">
+      <c r="M20" s="24" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N20" s="16"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B21" s="21"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="11" t="str" cm="1">
-        <f t="array" ref="C21">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B21,"SP_PRICE_CLOSE",WORKDAY(#REF!+1,-1),"Options: NA=NA")</f>
-        <v>#PEND</v>
+        <f t="array" ref="C21">_xll.SNL.Clients.Office.Excel.Functions.SPG("$"&amp;$H$2&amp;$B21,"SP_PRICE_CLOSE",WORKDAY(E21+1,-1),"Options: NA=NA")</f>
+        <v>#INVALID FUNCTION PARAMETER</v>
       </c>
       <c r="E21" s="13"/>
       <c r="F21" s="14"/>
       <c r="G21" s="14"/>
       <c r="H21" s="15"/>
-      <c r="I21" s="30"/>
-      <c r="J21" s="23"/>
-      <c r="K21" s="23"/>
-      <c r="L21" s="25" t="str">
+      <c r="I21" s="29"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="24" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M21" s="25" t="str">
+      <c r="M21" s="24" t="str">
         <f t="shared" si="1"/>
         <v xml:space="preserve">n/a </v>
       </c>
       <c r="N21" s="16"/>
     </row>
     <row r="22" spans="2:14" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I22" s="31"/>
+      <c r="I22" s="30"/>
     </row>
     <row r="23" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E23" s="26" t="s">
+      <c r="E23" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="32"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
-      <c r="L23" s="28" t="str">
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="26"/>
+      <c r="L23" s="27" t="str">
         <f>IFERROR(AVERAGE(L7:L21),"n/a ")</f>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="M23" s="28" t="str">
+      <c r="M23" s="27" t="str">
         <f>IFERROR(AVERAGE(M7:M21),"n/a ")</f>
         <v xml:space="preserve">n/a </v>
       </c>
-      <c r="N23" s="26"/>
+      <c r="N23" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>